<commit_message>
Rebuild forecast ranges on EWMA volatility and fix recent-period scoring
- Ranges now scale by 10-day-half-life EWMA volatility: same coverage in the
  2018-2026 backtest, 2-5% narrower ranges
- Last-2-year metrics calibrate bands on full history before restricting to
  the period (previously re-calibrated inside the window, understating
  coverage as 72-77% when it is ~78-85%)
- Excel Details sheet adds last-2-year 80% hit rate and a readable data label
- Refreshed sample_run_2026-09-22 outputs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F5xXFPuQBuXBKUV8bo8d9G
</commit_message>
<xml_diff>
--- a/price_forecast/sample_run_2026-09-22/oil_gas_price_forecast.xlsx
+++ b/price_forecast/sample_run_2026-09-22/oil_gas_price_forecast.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
   <si>
     <t xml:space="preserve">Crude oil Price forecast per bbl</t>
   </si>
@@ -110,6 +110,9 @@
     <t xml:space="preserve">80% range hit rate</t>
   </si>
   <si>
+    <t xml:space="preserve">80% range hit rate, last 2 yrs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Model used</t>
   </si>
   <si>
@@ -128,7 +131,7 @@
     <t xml:space="preserve">Ridge regression</t>
   </si>
   <si>
-    <t xml:space="preserve">Data: EIA daily spot prices (GitHub mirror of EIA data), to 2026-09-22. Blue = model output (python run_forecast.py); black = formula.</t>
+    <t xml:space="preserve">Data: EIA daily spot prices (github.com/datasets mirror). Blue = model output (python run_forecast.py); black = formula.</t>
   </si>
   <si>
     <t xml:space="preserve">% accuracy = 1 - backtest mean absolute % error of the forecast price (8-year walk-forward, out-of-sample).</t>
@@ -681,19 +684,19 @@
       </c>
       <c r="H18" s="5" t="n">
         <f aca="false">Details!G6</f>
-        <v>2.80272144506248</v>
+        <v>2.80654604018657</v>
       </c>
       <c r="I18" s="6" t="n">
         <f aca="false">Details!O6</f>
-        <v>0.894937203237807</v>
+        <v>0.895092240708954</v>
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
-        <v>2.80340417020803</v>
+        <v>2.80886934185562</v>
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
-        <v>0.856720549778292</v>
+        <v>0.856240258248329</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -732,7 +735,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -745,7 +748,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -803,13 +807,16 @@
       <c r="R1" s="3" t="s">
         <v>28</v>
       </c>
+      <c r="S1" s="3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>7</v>
@@ -831,16 +838,16 @@
         <v>0</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>101.925126707675</v>
+        <v>101.94825056334</v>
       </c>
       <c r="J2" s="11" t="n">
-        <v>128.623078832282</v>
+        <v>128.565264790535</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>91.8907034632722</v>
+        <v>93.1144400399458</v>
       </c>
       <c r="L2" s="11" t="n">
-        <v>137.761906515218</v>
+        <v>137.225317462959</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>0.531219980787704</v>
@@ -856,10 +863,13 @@
         <v>0.6940441882805</v>
       </c>
       <c r="Q2" s="13" t="n">
-        <v>0.792008757525999</v>
-      </c>
-      <c r="R2" s="16" t="s">
-        <v>30</v>
+        <v>0.789272030651341</v>
+      </c>
+      <c r="R2" s="13" t="n">
+        <v>0.787234042553192</v>
+      </c>
+      <c r="S2" s="16" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -867,7 +877,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3" s="9" t="n">
         <v>15</v>
@@ -889,16 +899,16 @@
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>95.0654871708784</v>
+        <v>95.509259484221</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>135.603960740583</v>
+        <v>135.762660795561</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>82.3148025556315</v>
+        <v>82.6121811734834</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>151.889329853362</v>
+        <v>153.35805542599</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>0.547687861271676</v>
@@ -914,10 +924,13 @@
         <v>0.533718689788054</v>
       </c>
       <c r="Q3" s="13" t="n">
-        <v>0.792286501377411</v>
-      </c>
-      <c r="R3" s="16" t="s">
-        <v>30</v>
+        <v>0.79504132231405</v>
+      </c>
+      <c r="R3" s="13" t="n">
+        <v>0.778864970645792</v>
+      </c>
+      <c r="S3" s="16" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -925,7 +938,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>7</v>
@@ -947,16 +960,16 @@
         <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>88.3597279676689</v>
+        <v>88.5392064656678</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>104.236602534808</v>
+        <v>104.172170454986</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>81.8919952620275</v>
+        <v>82.864404203947</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>108.889196172455</v>
+        <v>108.594045600806</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>0.535542747358309</v>
@@ -972,10 +985,13 @@
         <v>0.700768491834774</v>
       </c>
       <c r="Q4" s="13" t="n">
-        <v>0.79912424740011</v>
-      </c>
-      <c r="R4" s="16" t="s">
-        <v>30</v>
+        <v>0.802408319649699</v>
+      </c>
+      <c r="R4" s="13" t="n">
+        <v>0.808510638297872</v>
+      </c>
+      <c r="S4" s="16" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -983,7 +999,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>15</v>
@@ -1005,16 +1021,16 @@
         <v>0</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>84.5039939726771</v>
+        <v>84.7446636495265</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>107.69485492397</v>
+        <v>107.725208886862</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>75.7511186524678</v>
+        <v>76.4697250875054</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>116.169820720737</v>
+        <v>116.156894768211</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>0.554913294797688</v>
@@ -1030,18 +1046,21 @@
         <v>0.534200385356455</v>
       </c>
       <c r="Q5" s="13" t="n">
-        <v>0.813774104683196</v>
-      </c>
-      <c r="R5" s="16" t="s">
-        <v>30</v>
+        <v>0.808264462809917</v>
+      </c>
+      <c r="R5" s="13" t="n">
+        <v>0.812133072407045</v>
+      </c>
+      <c r="S5" s="16" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>7</v>
@@ -1056,50 +1075,53 @@
         <v>2.9</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>2.80272144506248</v>
+        <v>2.80654604018657</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">G6/F6-1</f>
-        <v>-0.0335443292888015</v>
+        <v>-0.0322255033839421</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>2.6056409557349</v>
+        <v>2.62490595894122</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>3.09000841299767</v>
+        <v>3.05537321171659</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>2.46457089258487</v>
+        <v>2.49426858013911</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>3.40735253094568</v>
+        <v>3.25419923927638</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>0.299231508165226</v>
+        <v>0.286743515850144</v>
       </c>
       <c r="N6" s="14" t="n">
-        <v>0.105062796762193</v>
+        <v>0.104907759291046</v>
       </c>
       <c r="O6" s="15" t="n">
         <f aca="false">1-N6</f>
-        <v>0.894937203237807</v>
+        <v>0.895092240708954</v>
       </c>
       <c r="P6" s="13" t="n">
-        <v>0.368395773294909</v>
+        <v>0.373198847262248</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.83032293377121</v>
-      </c>
-      <c r="R6" s="16" t="s">
-        <v>33</v>
+        <v>0.82703886152162</v>
+      </c>
+      <c r="R6" s="13" t="n">
+        <v>0.851063829787234</v>
+      </c>
+      <c r="S6" s="16" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>15</v>
@@ -1114,62 +1136,65 @@
         <v>2.9</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>2.80340417020803</v>
+        <v>2.80886934185562</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/F7-1</f>
-        <v>-0.0333089068248189</v>
+        <v>-0.0314243648773711</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.52402282831474</v>
+        <v>2.55387828058093</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.23201443704406</v>
+        <v>3.17532165595327</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.33290566134017</v>
+        <v>2.3958894745275</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.90079026686491</v>
+        <v>3.54950158221099</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.335260115606936</v>
+        <v>0.329479768786127</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>0.143279450221708</v>
+        <v>0.143759741751671</v>
       </c>
       <c r="O7" s="15" t="n">
         <f aca="false">1-N7</f>
-        <v>0.856720549778292</v>
+        <v>0.856240258248329</v>
       </c>
       <c r="P7" s="13" t="n">
-        <v>0.271676300578035</v>
+        <v>0.263969171483622</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0.83030303030303</v>
-      </c>
-      <c r="R7" s="16" t="s">
-        <v>33</v>
+        <v>0.830853994490358</v>
+      </c>
+      <c r="R7" s="13" t="n">
+        <v>0.831702544031311</v>
+      </c>
+      <c r="S7" s="16" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>